<commit_message>
Completed redux + next.js
</commit_message>
<xml_diff>
--- a/Nextjs_Redux_Migration_Plan.xlsx
+++ b/Nextjs_Redux_Migration_Plan.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +40,17 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00006100"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +67,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
         <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -87,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -100,6 +119,10 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -465,13 +488,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -495,6 +519,11 @@
           <t>Remarks</t>
         </is>
       </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -513,6 +542,11 @@
           <t>Create frontend app alongside existing time-tracker-backend; configure ESLint/Prettier and folder structure (app/, components/, features/).</t>
         </is>
       </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -531,6 +565,11 @@
           <t>Set up store.ts, root reducer, typed hooks (useAppDispatch/useAppSelector), and wrap app in &lt;Provider&gt; via a client-side layout wrapper.</t>
         </is>
       </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -549,6 +588,11 @@
           <t>Base URL config via env vars (NEXT_PUBLIC_API_URL), Axios instance, and typed request helpers matching API.md endpoints for Project/Task/State.</t>
         </is>
       </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -567,6 +611,11 @@
           <t>CRUD thunks for GET/POST/PUT/DELETE /Project; loading/error state handling.</t>
         </is>
       </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -585,6 +634,11 @@
           <t>CRUD + PATCH thunks for /Task, plus parent/nested task fetch endpoints (/Task/parent/{projectId}, /Task/nested/{parentTaskId}).</t>
         </is>
       </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -603,6 +657,11 @@
           <t>CRUD thunks for /State; used to drive task status columns.</t>
         </is>
       </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -621,6 +680,11 @@
           <t>Route: /projects - list, create, edit, delete projects; links into project detail/task board.</t>
         </is>
       </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -639,6 +703,11 @@
           <t>Integrate TipTap for description field (HTML) per API.md rich-text contract; connect to projectsSlice.</t>
         </is>
       </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -657,6 +726,11 @@
           <t>Route: /projects/[id] - render parent tasks and expandable nested subtasks using tasksSlice selectors.</t>
         </is>
       </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -675,6 +749,11 @@
           <t>TipTap-based description editor for tasks; supports parentID selection and projectID association.</t>
         </is>
       </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -693,6 +772,11 @@
           <t>Group tasks by stateID into columns (Pending/In Progress/etc.) sourced from statesSlice; improves on current flat list.</t>
         </is>
       </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -711,6 +795,11 @@
           <t>Use dnd-kit to move tasks between state columns, dispatching PATCH /Task/{id} on drop.</t>
         </is>
       </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -729,6 +818,11 @@
           <t>Start/stop timer UI per task that accumulates into timeTaken and PATCHes the backend on stop.</t>
         </is>
       </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="2" t="n">
@@ -747,6 +841,11 @@
           <t>Base styling, theme tokens, and shared layout components for consistent UI.</t>
         </is>
       </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -765,6 +864,11 @@
           <t>Toast notifications, skeleton loaders, and error boundaries wired to Redux async states.</t>
         </is>
       </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -783,6 +887,11 @@
           <t>next.config.js, .env.example, CORS check against ASP.NET backend, and README update for running both apps together.</t>
         </is>
       </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -799,6 +908,11 @@
       <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Run app against local backend; verify project/task CRUD, drag-and-drop, and timer flows end-to-end.</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>